<commit_message>
update test result for empirical verification of experts +  fix training script
</commit_message>
<xml_diff>
--- a/paper/test_results.xlsx
+++ b/paper/test_results.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Mixture-of-Experts_Research\paper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D058737F-6797-4850-BE41-202350495F45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F81F083-49FD-4FA8-9465-44F36FC8F5AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-86" yWindow="0" windowWidth="16629" windowHeight="17880" activeTab="1" xr2:uid="{7F82E78F-F225-4B75-B204-CA5D83064DD0}"/>
+    <workbookView xWindow="74355" yWindow="0" windowWidth="12150" windowHeight="15585" xr2:uid="{7F82E78F-F225-4B75-B204-CA5D83064DD0}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Empirical_Results_Experts" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -228,6 +228,10 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -238,15 +242,11 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -581,6 +581,398 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF7419F7-AE6D-458E-87E6-B4E28D246AFC}">
+  <dimension ref="A2:H25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="3" max="3" width="13.84375" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="13.3046875" customWidth="1"/>
+    <col min="6" max="6" width="14.61328125" customWidth="1"/>
+    <col min="7" max="7" width="9.23046875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="C2" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="14"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A3" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A4" s="18"/>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" s="3">
+        <v>0.99209999999999998</v>
+      </c>
+      <c r="D4" s="3">
+        <v>0.58819999999999995</v>
+      </c>
+      <c r="E4" s="3">
+        <v>0.84</v>
+      </c>
+      <c r="F4" s="3">
+        <v>1E-4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A5" s="18"/>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" s="3">
+        <v>0.99270000000000003</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0.43640000000000001</v>
+      </c>
+      <c r="E5" s="3">
+        <v>0.83879999999999999</v>
+      </c>
+      <c r="F5" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A6" s="18"/>
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="C6" s="3">
+        <v>0.99199999999999999</v>
+      </c>
+      <c r="D6" s="3">
+        <v>0.4244</v>
+      </c>
+      <c r="E6" s="3">
+        <v>0.83550000000000002</v>
+      </c>
+      <c r="F6" s="3">
+        <v>2.0000000000000001E-4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A7" s="18"/>
+      <c r="B7">
+        <v>4</v>
+      </c>
+      <c r="C7" s="3">
+        <v>0.99150000000000005</v>
+      </c>
+      <c r="D7" s="3">
+        <v>0.39140000000000003</v>
+      </c>
+      <c r="E7" s="3">
+        <v>0.83789999999999998</v>
+      </c>
+      <c r="F7" s="3">
+        <v>1E-4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A8" s="18"/>
+      <c r="B8">
+        <v>5</v>
+      </c>
+      <c r="C8" s="3">
+        <v>0.99099999999999999</v>
+      </c>
+      <c r="D8" s="3">
+        <v>0.46250000000000002</v>
+      </c>
+      <c r="E8" s="3">
+        <v>0.83530000000000004</v>
+      </c>
+      <c r="F8" s="3">
+        <v>1E-4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A9" s="18"/>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="13">
+        <f>AVERAGE(C4:C8)</f>
+        <v>0.99185999999999996</v>
+      </c>
+      <c r="D9" s="13">
+        <f t="shared" ref="D9:F9" si="0">AVERAGE(D4:D8)</f>
+        <v>0.46057999999999993</v>
+      </c>
+      <c r="E9" s="13">
+        <f t="shared" si="0"/>
+        <v>0.83750000000000002</v>
+      </c>
+      <c r="F9" s="13">
+        <f t="shared" si="0"/>
+        <v>1E-4</v>
+      </c>
+      <c r="H9" s="3">
+        <f>C9-D9</f>
+        <v>0.53127999999999997</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A10" s="18"/>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="13">
+        <f>_xlfn.STDEV.S(C4:C8)</f>
+        <v>6.4265076052238772E-4</v>
+      </c>
+      <c r="D10" s="13">
+        <f t="shared" ref="D10:F10" si="1">_xlfn.STDEV.S(D4:D8)</f>
+        <v>7.5779429926597017E-2</v>
+      </c>
+      <c r="E10" s="13">
+        <f t="shared" si="1"/>
+        <v>2.0579115627256395E-3</v>
+      </c>
+      <c r="F10" s="13">
+        <f t="shared" si="1"/>
+        <v>7.0710678118654754E-5</v>
+      </c>
+      <c r="H10" s="3">
+        <f>E9-F9</f>
+        <v>0.83740000000000003</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="C11" t="str">
+        <f>TEXT(C9,"0.00%") &amp; " ± " &amp; TEXT(C10,"0.00%")</f>
+        <v>99.19% ± 0.06%</v>
+      </c>
+      <c r="D11" t="str">
+        <f>TEXT(D9,"0.00%") &amp; " ± " &amp; TEXT(D10,"0.00%")</f>
+        <v>46.06% ± 7.58%</v>
+      </c>
+      <c r="E11" t="str">
+        <f>TEXT(E9,"0.00%") &amp; " ± " &amp; TEXT(E10,"0.00%")</f>
+        <v>83.75% ± 0.21%</v>
+      </c>
+      <c r="F11" t="str">
+        <f>TEXT(F9,"0.00%") &amp; " ± " &amp; TEXT(F10,"0.00%")</f>
+        <v>0.01% ± 0.01%</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A13" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A14" s="18"/>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" s="3">
+        <v>0.99170000000000003</v>
+      </c>
+      <c r="D14" s="3">
+        <v>0.92849999999999999</v>
+      </c>
+      <c r="E14" s="3">
+        <v>0.77800000000000002</v>
+      </c>
+      <c r="F14" s="3">
+        <v>0.17269999999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A15" s="18"/>
+      <c r="B15">
+        <v>2</v>
+      </c>
+      <c r="C15" s="3">
+        <v>0.99119999999999997</v>
+      </c>
+      <c r="D15" s="3">
+        <v>0.81410000000000005</v>
+      </c>
+      <c r="E15" s="3">
+        <v>0.77229999999999999</v>
+      </c>
+      <c r="F15" s="3">
+        <v>0.1719</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A16" s="18"/>
+      <c r="B16">
+        <v>3</v>
+      </c>
+      <c r="C16" s="3">
+        <v>0.9919</v>
+      </c>
+      <c r="D16" s="3">
+        <v>0.92369999999999997</v>
+      </c>
+      <c r="E16" s="3">
+        <v>0.77310000000000001</v>
+      </c>
+      <c r="F16" s="3">
+        <v>0.17199999999999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A17" s="18"/>
+      <c r="B17">
+        <v>4</v>
+      </c>
+      <c r="C17" s="3">
+        <v>0.99150000000000005</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0.9556</v>
+      </c>
+      <c r="E17" s="3">
+        <v>0.77590000000000003</v>
+      </c>
+      <c r="F17" s="3">
+        <v>0.17660000000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A18" s="18"/>
+      <c r="B18">
+        <v>5</v>
+      </c>
+      <c r="C18" s="3">
+        <v>0.99199999999999999</v>
+      </c>
+      <c r="D18" s="3">
+        <v>0.91669999999999996</v>
+      </c>
+      <c r="E18" s="3">
+        <v>0.77769999999999995</v>
+      </c>
+      <c r="F18" s="3">
+        <v>0.16900000000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A19" s="18"/>
+      <c r="B19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" s="13">
+        <f>AVERAGE(C14:C18)</f>
+        <v>0.9916600000000001</v>
+      </c>
+      <c r="D19" s="13">
+        <f t="shared" ref="D19" si="2">AVERAGE(D14:D18)</f>
+        <v>0.90771999999999997</v>
+      </c>
+      <c r="E19" s="13">
+        <f t="shared" ref="E19" si="3">AVERAGE(E14:E18)</f>
+        <v>0.77539999999999998</v>
+      </c>
+      <c r="F19" s="13">
+        <f t="shared" ref="F19" si="4">AVERAGE(F14:F18)</f>
+        <v>0.17243999999999998</v>
+      </c>
+      <c r="H19" s="3">
+        <f>C19-D19</f>
+        <v>8.3940000000000126E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A20" s="18"/>
+      <c r="B20" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" s="13">
+        <f>_xlfn.STDEV.S(C14:C18)</f>
+        <v>3.2093613071762869E-4</v>
+      </c>
+      <c r="D20" s="13">
+        <f t="shared" ref="D20:F20" si="5">_xlfn.STDEV.S(D14:D18)</f>
+        <v>5.4371426319345321E-2</v>
+      </c>
+      <c r="E20" s="13">
+        <f t="shared" si="5"/>
+        <v>2.6076809620810574E-3</v>
+      </c>
+      <c r="F20" s="13">
+        <f t="shared" si="5"/>
+        <v>2.7245183060497129E-3</v>
+      </c>
+      <c r="H20" s="3">
+        <f>E19-F19</f>
+        <v>0.60295999999999994</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="C21" t="str">
+        <f>TEXT(C19,"0.00%") &amp; " ± " &amp; TEXT(C20,"0.00%")</f>
+        <v>99.17% ± 0.03%</v>
+      </c>
+      <c r="D21" t="str">
+        <f t="shared" ref="D21:F21" si="6">TEXT(D19,"0.00%") &amp; " ± " &amp; TEXT(D20,"0.00%")</f>
+        <v>90.77% ± 5.44%</v>
+      </c>
+      <c r="E21" t="str">
+        <f t="shared" si="6"/>
+        <v>77.54% ± 0.26%</v>
+      </c>
+      <c r="F21" t="str">
+        <f t="shared" si="6"/>
+        <v>17.24% ± 0.27%</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="C25" s="3"/>
+      <c r="E25" s="3"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="A3:A10"/>
+    <mergeCell ref="A13:A20"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{298A52AC-B951-4303-84A2-1510182D5632}">
   <dimension ref="A2:N47"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
@@ -593,22 +985,22 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="B2" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="16" t="s">
+      <c r="B2" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16" t="s">
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="B3" s="18"/>
+      <c r="B3" s="19"/>
       <c r="D3" t="s">
         <v>1</v>
       </c>
@@ -635,10 +1027,10 @@
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="15">
         <v>7.8399999999999997E-3</v>
       </c>
       <c r="C4" s="2">
@@ -673,8 +1065,8 @@
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="A5" s="14"/>
-      <c r="B5" s="14"/>
+      <c r="A5" s="16"/>
+      <c r="B5" s="16"/>
       <c r="C5" s="4">
         <v>2</v>
       </c>
@@ -707,8 +1099,8 @@
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="A6" s="14"/>
-      <c r="B6" s="14"/>
+      <c r="A6" s="16"/>
+      <c r="B6" s="16"/>
       <c r="C6" s="4">
         <v>3</v>
       </c>
@@ -741,8 +1133,8 @@
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="A7" s="14"/>
-      <c r="B7" s="14"/>
+      <c r="A7" s="16"/>
+      <c r="B7" s="16"/>
       <c r="C7" s="4">
         <v>4</v>
       </c>
@@ -775,8 +1167,8 @@
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="A8" s="14"/>
-      <c r="B8" s="14"/>
+      <c r="A8" s="16"/>
+      <c r="B8" s="16"/>
       <c r="C8" s="4">
         <v>5</v>
       </c>
@@ -809,8 +1201,8 @@
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="A9" s="14"/>
-      <c r="B9" s="15"/>
+      <c r="A9" s="16"/>
+      <c r="B9" s="17"/>
       <c r="C9" s="8" t="s">
         <v>8</v>
       </c>
@@ -848,8 +1240,8 @@
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="A10" s="14"/>
-      <c r="B10" s="13">
+      <c r="A10" s="16"/>
+      <c r="B10" s="15">
         <v>1.5689999999999999E-2</v>
       </c>
       <c r="C10" s="2">
@@ -890,8 +1282,8 @@
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="A11" s="14"/>
-      <c r="B11" s="14"/>
+      <c r="A11" s="16"/>
+      <c r="B11" s="16"/>
       <c r="C11" s="4">
         <v>2</v>
       </c>
@@ -924,8 +1316,8 @@
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="A12" s="14"/>
-      <c r="B12" s="14"/>
+      <c r="A12" s="16"/>
+      <c r="B12" s="16"/>
       <c r="C12" s="4">
         <v>3</v>
       </c>
@@ -958,8 +1350,8 @@
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="A13" s="14"/>
-      <c r="B13" s="14"/>
+      <c r="A13" s="16"/>
+      <c r="B13" s="16"/>
       <c r="C13" s="4">
         <v>4</v>
       </c>
@@ -992,8 +1384,8 @@
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="A14" s="14"/>
-      <c r="B14" s="14"/>
+      <c r="A14" s="16"/>
+      <c r="B14" s="16"/>
       <c r="C14" s="4">
         <v>5</v>
       </c>
@@ -1026,8 +1418,8 @@
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="A15" s="14"/>
-      <c r="B15" s="15"/>
+      <c r="A15" s="16"/>
+      <c r="B15" s="17"/>
       <c r="C15" s="8" t="s">
         <v>8</v>
       </c>
@@ -1065,8 +1457,8 @@
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="A16" s="14"/>
-      <c r="B16" s="13">
+      <c r="A16" s="16"/>
+      <c r="B16" s="15">
         <v>3.1370000000000002E-2</v>
       </c>
       <c r="C16" s="2">
@@ -1101,8 +1493,8 @@
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A17" s="14"/>
-      <c r="B17" s="14"/>
+      <c r="A17" s="16"/>
+      <c r="B17" s="16"/>
       <c r="C17" s="4">
         <v>2</v>
       </c>
@@ -1135,8 +1527,8 @@
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A18" s="14"/>
-      <c r="B18" s="14"/>
+      <c r="A18" s="16"/>
+      <c r="B18" s="16"/>
       <c r="C18" s="4">
         <v>3</v>
       </c>
@@ -1169,8 +1561,8 @@
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A19" s="14"/>
-      <c r="B19" s="14"/>
+      <c r="A19" s="16"/>
+      <c r="B19" s="16"/>
       <c r="C19" s="4">
         <v>4</v>
       </c>
@@ -1203,8 +1595,8 @@
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A20" s="14"/>
-      <c r="B20" s="14"/>
+      <c r="A20" s="16"/>
+      <c r="B20" s="16"/>
       <c r="C20" s="4">
         <v>5</v>
       </c>
@@ -1237,8 +1629,8 @@
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A21" s="15"/>
-      <c r="B21" s="15"/>
+      <c r="A21" s="17"/>
+      <c r="B21" s="17"/>
       <c r="C21" s="8" t="s">
         <v>8</v>
       </c>
@@ -1387,10 +1779,10 @@
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A27" s="13" t="s">
+      <c r="A27" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="B27" s="13">
+      <c r="B27" s="15">
         <v>7.8399999999999997E-3</v>
       </c>
       <c r="C27" s="2">
@@ -1425,8 +1817,8 @@
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A28" s="14"/>
-      <c r="B28" s="14"/>
+      <c r="A28" s="16"/>
+      <c r="B28" s="16"/>
       <c r="C28" s="4">
         <v>2</v>
       </c>
@@ -1459,8 +1851,8 @@
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A29" s="14"/>
-      <c r="B29" s="14"/>
+      <c r="A29" s="16"/>
+      <c r="B29" s="16"/>
       <c r="C29" s="4">
         <v>3</v>
       </c>
@@ -1493,8 +1885,8 @@
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A30" s="14"/>
-      <c r="B30" s="14"/>
+      <c r="A30" s="16"/>
+      <c r="B30" s="16"/>
       <c r="C30" s="4">
         <v>4</v>
       </c>
@@ -1527,8 +1919,8 @@
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A31" s="14"/>
-      <c r="B31" s="14"/>
+      <c r="A31" s="16"/>
+      <c r="B31" s="16"/>
       <c r="C31" s="4">
         <v>5</v>
       </c>
@@ -1561,8 +1953,8 @@
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A32" s="14"/>
-      <c r="B32" s="15"/>
+      <c r="A32" s="16"/>
+      <c r="B32" s="17"/>
       <c r="C32" s="8" t="s">
         <v>8</v>
       </c>
@@ -1600,8 +1992,8 @@
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A33" s="14"/>
-      <c r="B33" s="13">
+      <c r="A33" s="16"/>
+      <c r="B33" s="15">
         <v>1.5689999999999999E-2</v>
       </c>
       <c r="C33" s="2">
@@ -1636,8 +2028,8 @@
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A34" s="14"/>
-      <c r="B34" s="14"/>
+      <c r="A34" s="16"/>
+      <c r="B34" s="16"/>
       <c r="C34" s="4">
         <v>2</v>
       </c>
@@ -1670,8 +2062,8 @@
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A35" s="14"/>
-      <c r="B35" s="14"/>
+      <c r="A35" s="16"/>
+      <c r="B35" s="16"/>
       <c r="C35" s="4">
         <v>3</v>
       </c>
@@ -1704,8 +2096,8 @@
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A36" s="14"/>
-      <c r="B36" s="14"/>
+      <c r="A36" s="16"/>
+      <c r="B36" s="16"/>
       <c r="C36" s="4">
         <v>4</v>
       </c>
@@ -1738,8 +2130,8 @@
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A37" s="14"/>
-      <c r="B37" s="14"/>
+      <c r="A37" s="16"/>
+      <c r="B37" s="16"/>
       <c r="C37" s="4">
         <v>5</v>
       </c>
@@ -1772,8 +2164,8 @@
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A38" s="14"/>
-      <c r="B38" s="15"/>
+      <c r="A38" s="16"/>
+      <c r="B38" s="17"/>
       <c r="C38" s="8" t="s">
         <v>8</v>
       </c>
@@ -1811,8 +2203,8 @@
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A39" s="14"/>
-      <c r="B39" s="13">
+      <c r="A39" s="16"/>
+      <c r="B39" s="15">
         <v>3.1370000000000002E-2</v>
       </c>
       <c r="C39" s="2">
@@ -1847,8 +2239,8 @@
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A40" s="14"/>
-      <c r="B40" s="14"/>
+      <c r="A40" s="16"/>
+      <c r="B40" s="16"/>
       <c r="C40" s="4">
         <v>2</v>
       </c>
@@ -1881,8 +2273,8 @@
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A41" s="14"/>
-      <c r="B41" s="14"/>
+      <c r="A41" s="16"/>
+      <c r="B41" s="16"/>
       <c r="C41" s="4">
         <v>3</v>
       </c>
@@ -1915,8 +2307,8 @@
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A42" s="14"/>
-      <c r="B42" s="14"/>
+      <c r="A42" s="16"/>
+      <c r="B42" s="16"/>
       <c r="C42" s="4">
         <v>4</v>
       </c>
@@ -1949,8 +2341,8 @@
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A43" s="14"/>
-      <c r="B43" s="14"/>
+      <c r="A43" s="16"/>
+      <c r="B43" s="16"/>
       <c r="C43" s="4">
         <v>5</v>
       </c>
@@ -1983,8 +2375,8 @@
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A44" s="15"/>
-      <c r="B44" s="15"/>
+      <c r="A44" s="17"/>
+      <c r="B44" s="17"/>
       <c r="C44" s="8" t="s">
         <v>8</v>
       </c>
@@ -2134,402 +2526,19 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A4:A21"/>
+    <mergeCell ref="A27:A44"/>
+    <mergeCell ref="B27:B32"/>
+    <mergeCell ref="B33:B38"/>
+    <mergeCell ref="B39:B44"/>
     <mergeCell ref="D2:F2"/>
     <mergeCell ref="G2:I2"/>
     <mergeCell ref="B4:B9"/>
     <mergeCell ref="B10:B15"/>
     <mergeCell ref="B16:B21"/>
     <mergeCell ref="B2:B3"/>
-    <mergeCell ref="A4:A21"/>
-    <mergeCell ref="A27:A44"/>
-    <mergeCell ref="B27:B32"/>
-    <mergeCell ref="B33:B38"/>
-    <mergeCell ref="B39:B44"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" verticalDpi="0" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF7419F7-AE6D-458E-87E6-B4E28D246AFC}">
-  <dimension ref="A2:H21"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
-  <cols>
-    <col min="3" max="3" width="13.84375" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="13.3046875" customWidth="1"/>
-    <col min="6" max="6" width="14.61328125" customWidth="1"/>
-    <col min="7" max="7" width="9.23046875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A3" s="17" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A4" s="17"/>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4" s="3">
-        <v>0.99099999999999999</v>
-      </c>
-      <c r="D4" s="3">
-        <v>0.47189999999999999</v>
-      </c>
-      <c r="E4" s="3">
-        <v>0.84099999999999997</v>
-      </c>
-      <c r="F4" s="3">
-        <v>1E-4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A5" s="17"/>
-      <c r="B5">
-        <v>2</v>
-      </c>
-      <c r="C5" s="3">
-        <v>0.99239999999999995</v>
-      </c>
-      <c r="D5" s="3">
-        <v>0.62019999999999997</v>
-      </c>
-      <c r="E5" s="3">
-        <v>0.83779999999999999</v>
-      </c>
-      <c r="F5" s="3">
-        <v>2.9999999999999997E-4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A6" s="17"/>
-      <c r="B6">
-        <v>3</v>
-      </c>
-      <c r="C6" s="3">
-        <v>0.99209999999999998</v>
-      </c>
-      <c r="D6" s="3">
-        <v>0.52569999999999995</v>
-      </c>
-      <c r="E6" s="3">
-        <v>0.83599999999999997</v>
-      </c>
-      <c r="F6" s="3">
-        <v>1E-4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A7" s="17"/>
-      <c r="B7">
-        <v>4</v>
-      </c>
-      <c r="C7" s="3">
-        <v>0.99139999999999995</v>
-      </c>
-      <c r="D7" s="3">
-        <v>0.53390000000000004</v>
-      </c>
-      <c r="E7" s="3">
-        <v>0.83750000000000002</v>
-      </c>
-      <c r="F7" s="3">
-        <v>1E-4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A8" s="17"/>
-      <c r="B8">
-        <v>5</v>
-      </c>
-      <c r="C8" s="3">
-        <v>0.99199999999999999</v>
-      </c>
-      <c r="D8" s="3">
-        <v>0.60709999999999997</v>
-      </c>
-      <c r="E8" s="3">
-        <v>0.83799999999999997</v>
-      </c>
-      <c r="F8" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A9" s="17"/>
-      <c r="B9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" s="19">
-        <f>AVERAGE(C4:C8)</f>
-        <v>0.99177999999999999</v>
-      </c>
-      <c r="D9" s="19">
-        <f t="shared" ref="D9:F9" si="0">AVERAGE(D4:D8)</f>
-        <v>0.55176000000000003</v>
-      </c>
-      <c r="E9" s="19">
-        <f t="shared" si="0"/>
-        <v>0.83805999999999992</v>
-      </c>
-      <c r="F9" s="19">
-        <f t="shared" si="0"/>
-        <v>1.2000000000000002E-4</v>
-      </c>
-      <c r="H9" s="3">
-        <f>C9-D9</f>
-        <v>0.44001999999999997</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A10" s="17"/>
-      <c r="B10" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" s="19">
-        <f>_xlfn.STDEV.S(C4:C8)</f>
-        <v>5.6745043836443855E-4</v>
-      </c>
-      <c r="D10" s="19">
-        <f t="shared" ref="D10:F10" si="1">_xlfn.STDEV.S(D4:D8)</f>
-        <v>6.1486323682588141E-2</v>
-      </c>
-      <c r="E10" s="19">
-        <f t="shared" si="1"/>
-        <v>1.8215378118501926E-3</v>
-      </c>
-      <c r="F10" s="19">
-        <f t="shared" si="1"/>
-        <v>1.0954451150103323E-4</v>
-      </c>
-      <c r="H10" s="3">
-        <f>E9-F9</f>
-        <v>0.83793999999999991</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="C11" t="str">
-        <f>TEXT(C9,"0.00%") &amp; " ± " &amp; TEXT(C10,"0.00%")</f>
-        <v>99.18% ± 0.06%</v>
-      </c>
-      <c r="D11" t="str">
-        <f>TEXT(D9,"0.00%") &amp; " ± " &amp; TEXT(D10,"0.00%")</f>
-        <v>55.18% ± 6.15%</v>
-      </c>
-      <c r="E11" t="str">
-        <f>TEXT(E9,"0.00%") &amp; " ± " &amp; TEXT(E10,"0.00%")</f>
-        <v>83.81% ± 0.18%</v>
-      </c>
-      <c r="F11" t="str">
-        <f>TEXT(F9,"0.00%") &amp; " ± " &amp; TEXT(F10,"0.00%")</f>
-        <v>0.01% ± 0.01%</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A13" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="C13" t="s">
-        <v>13</v>
-      </c>
-      <c r="D13" t="s">
-        <v>14</v>
-      </c>
-      <c r="E13" t="s">
-        <v>13</v>
-      </c>
-      <c r="F13" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A14" s="17"/>
-      <c r="B14">
-        <v>1</v>
-      </c>
-      <c r="C14" s="3">
-        <v>0.99150000000000005</v>
-      </c>
-      <c r="D14" s="3">
-        <v>0.87870000000000004</v>
-      </c>
-      <c r="E14" s="3">
-        <v>0.77580000000000005</v>
-      </c>
-      <c r="F14" s="3">
-        <v>0.1704</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A15" s="17"/>
-      <c r="B15">
-        <v>2</v>
-      </c>
-      <c r="C15" s="3">
-        <v>0.99070000000000003</v>
-      </c>
-      <c r="D15" s="3">
-        <v>0.94769999999999999</v>
-      </c>
-      <c r="E15" s="3">
-        <v>0.77559999999999996</v>
-      </c>
-      <c r="F15" s="3">
-        <v>0.17100000000000001</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A16" s="17"/>
-      <c r="B16">
-        <v>3</v>
-      </c>
-      <c r="C16" s="3">
-        <v>0.99060000000000004</v>
-      </c>
-      <c r="D16" s="3">
-        <v>0.94399999999999995</v>
-      </c>
-      <c r="E16" s="3">
-        <v>0.77669999999999995</v>
-      </c>
-      <c r="F16" s="3">
-        <v>0.17879999999999999</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A17" s="17"/>
-      <c r="B17">
-        <v>4</v>
-      </c>
-      <c r="C17" s="3">
-        <v>0.99139999999999995</v>
-      </c>
-      <c r="D17" s="3">
-        <v>0.96519999999999995</v>
-      </c>
-      <c r="E17" s="3">
-        <v>0.77839999999999998</v>
-      </c>
-      <c r="F17" s="3">
-        <v>0.16700000000000001</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A18" s="17"/>
-      <c r="B18">
-        <v>5</v>
-      </c>
-      <c r="C18" s="3">
-        <v>0.99209999999999998</v>
-      </c>
-      <c r="D18" s="3">
-        <v>0.87960000000000005</v>
-      </c>
-      <c r="E18" s="3">
-        <v>0.77659999999999996</v>
-      </c>
-      <c r="F18" s="3">
-        <v>0.16950000000000001</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A19" s="17"/>
-      <c r="B19" t="s">
-        <v>8</v>
-      </c>
-      <c r="C19" s="19">
-        <f>AVERAGE(C14:C18)</f>
-        <v>0.99126000000000014</v>
-      </c>
-      <c r="D19" s="19">
-        <f t="shared" ref="D19" si="2">AVERAGE(D14:D18)</f>
-        <v>0.92303999999999997</v>
-      </c>
-      <c r="E19" s="19">
-        <f t="shared" ref="E19" si="3">AVERAGE(E14:E18)</f>
-        <v>0.77661999999999998</v>
-      </c>
-      <c r="F19" s="19">
-        <f t="shared" ref="F19" si="4">AVERAGE(F14:F18)</f>
-        <v>0.17133999999999999</v>
-      </c>
-      <c r="H19" s="3">
-        <f>C19-D19</f>
-        <v>6.8220000000000169E-2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A20" s="17"/>
-      <c r="B20" t="s">
-        <v>12</v>
-      </c>
-      <c r="C20" s="19">
-        <f>_xlfn.STDEV.S(C14:C18)</f>
-        <v>6.1886993787061242E-4</v>
-      </c>
-      <c r="D20" s="19">
-        <f t="shared" ref="D20:F20" si="5">_xlfn.STDEV.S(D14:D18)</f>
-        <v>4.0859429756177415E-2</v>
-      </c>
-      <c r="E20" s="19">
-        <f t="shared" si="5"/>
-        <v>1.1054410884348315E-3</v>
-      </c>
-      <c r="F20" s="19">
-        <f t="shared" si="5"/>
-        <v>4.4404954678503973E-3</v>
-      </c>
-      <c r="H20" s="3">
-        <f>E19-F19</f>
-        <v>0.60528000000000004</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="C21" t="str">
-        <f>TEXT(C19,"0.00%") &amp; " ± " &amp; TEXT(C20,"0.00%")</f>
-        <v>99.13% ± 0.06%</v>
-      </c>
-      <c r="D21" t="str">
-        <f t="shared" ref="D21:F21" si="6">TEXT(D19,"0.00%") &amp; " ± " &amp; TEXT(D20,"0.00%")</f>
-        <v>92.30% ± 4.09%</v>
-      </c>
-      <c r="E21" t="str">
-        <f t="shared" si="6"/>
-        <v>77.66% ± 0.11%</v>
-      </c>
-      <c r="F21" t="str">
-        <f t="shared" si="6"/>
-        <v>17.13% ± 0.44%</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A3:A10"/>
-    <mergeCell ref="A13:A20"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
update results to paper + remove time column
</commit_message>
<xml_diff>
--- a/paper/test_results.xlsx
+++ b/paper/test_results.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Mixture-of-Experts_Research\paper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3161135-5DE9-4A97-905A-AA910B274FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{574AF23B-0E19-49D9-9C49-28C081F15084}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="1" xr2:uid="{7F82E78F-F225-4B75-B204-CA5D83064DD0}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{7F82E78F-F225-4B75-B204-CA5D83064DD0}"/>
   </bookViews>
   <sheets>
     <sheet name="Empirical Results Experts" sheetId="2" r:id="rId1"/>
-    <sheet name="Formal Results Router 1" sheetId="5" r:id="rId2"/>
+    <sheet name="Formal Results Router" sheetId="5" r:id="rId2"/>
     <sheet name="Formal Results Expert" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -1146,7 +1146,7 @@
         <v>20</v>
       </c>
       <c r="E6">
-        <f t="shared" ref="E5:E8" si="1">$N$10-D6-F6</f>
+        <f t="shared" ref="E6:E8" si="1">$N$10-D6-F6</f>
         <v>0</v>
       </c>
       <c r="F6">
@@ -2408,17 +2408,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A27:A44"/>
+    <mergeCell ref="B27:B32"/>
+    <mergeCell ref="B33:B38"/>
+    <mergeCell ref="B39:B44"/>
+    <mergeCell ref="B2:B3"/>
     <mergeCell ref="D2:F2"/>
     <mergeCell ref="G2:I2"/>
     <mergeCell ref="A4:A21"/>
     <mergeCell ref="B4:B9"/>
     <mergeCell ref="B10:B15"/>
     <mergeCell ref="B16:B21"/>
-    <mergeCell ref="A27:A44"/>
-    <mergeCell ref="B27:B32"/>
-    <mergeCell ref="B33:B38"/>
-    <mergeCell ref="B39:B44"/>
-    <mergeCell ref="B2:B3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3739,12 +3739,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A14:A18"/>
-    <mergeCell ref="C2:F2"/>
-    <mergeCell ref="H2:K2"/>
-    <mergeCell ref="A4:A8"/>
-    <mergeCell ref="C12:F12"/>
-    <mergeCell ref="H12:K12"/>
     <mergeCell ref="A54:A58"/>
     <mergeCell ref="C22:F22"/>
     <mergeCell ref="H22:K22"/>
@@ -3757,6 +3751,12 @@
     <mergeCell ref="A44:A48"/>
     <mergeCell ref="C52:F52"/>
     <mergeCell ref="H52:K52"/>
+    <mergeCell ref="A14:A18"/>
+    <mergeCell ref="C2:F2"/>
+    <mergeCell ref="H2:K2"/>
+    <mergeCell ref="A4:A8"/>
+    <mergeCell ref="C12:F12"/>
+    <mergeCell ref="H12:K12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>